<commit_message>
update: new .gitignore repository dependencies
</commit_message>
<xml_diff>
--- a/docs/ESO-docs/ESO-finanzas.xlsx
+++ b/docs/ESO-docs/ESO-finanzas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pablo/Documents/github/AstroGit-OS/docs/ESO-docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03505DA9-CC29-5548-BF19-A58A2A6AA055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF54AFB-B3DD-B74C-978B-D54A9C36315A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="600" windowWidth="27880" windowHeight="17400" xr2:uid="{7AF2B69F-C7B1-BF4D-9F57-34C5ABF7EC90}"/>
+    <workbookView xWindow="16900" yWindow="600" windowWidth="11900" windowHeight="17400" xr2:uid="{7AF2B69F-C7B1-BF4D-9F57-34C5ABF7EC90}"/>
   </bookViews>
   <sheets>
     <sheet name="Componente" sheetId="1" r:id="rId1"/>
@@ -228,10 +228,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0;[Red]&quot;$&quot;\-#,##0"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -271,6 +272,12 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Palatino Linotype"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Palatino"/>
       <family val="1"/>
     </font>
   </fonts>
@@ -370,7 +377,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -455,6 +462,11 @@
     <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="6" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE0A9E87-FEB0-C341-B5E9-BA6B52C4C0B0}">
-  <dimension ref="B2:F10"/>
+  <dimension ref="B2:F37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
@@ -953,6 +965,113 @@
         <f>SUM(F3:F9)</f>
         <v>34950000</v>
       </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="33"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="33"/>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+    </row>
+    <row r="18" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="33"/>
+    </row>
+    <row r="19" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="33"/>
+    </row>
+    <row r="20" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="33"/>
+    </row>
+    <row r="21" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="33"/>
+    </row>
+    <row r="22" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="33"/>
+    </row>
+    <row r="23" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="33"/>
+    </row>
+    <row r="24" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="33"/>
+    </row>
+    <row r="25" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+    </row>
+    <row r="26" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="F26" s="33"/>
+    </row>
+    <row r="30" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="D30" s="32"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="33"/>
+    </row>
+    <row r="31" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="D31" s="32"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="33"/>
+    </row>
+    <row r="32" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="D32" s="32"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="33"/>
+    </row>
+    <row r="33" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D33" s="32"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="33"/>
+    </row>
+    <row r="34" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D34" s="32"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="33"/>
+    </row>
+    <row r="35" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D35" s="32"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="33"/>
+    </row>
+    <row r="36" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D36" s="32"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="33"/>
+    </row>
+    <row r="37" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="F37" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>